<commit_message>
Datos transaccionales: agrega oct-2026 (OC hasta el 23-10) y actualiza sep-2026 con la descarga del 24-10
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/administracion-y-entrega-de-beneficios/sep-2026.xlsx
+++ b/docs/oc-mensuales/administracion-y-entrega-de-beneficios/sep-2026.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M397"/>
+  <dimension ref="A1:M396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -4629,7 +4629,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -5084,7 +5084,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -5929,7 +5929,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -6319,7 +6319,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -8334,7 +8334,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -8919,7 +8919,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -9374,7 +9374,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -10349,7 +10349,7 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
@@ -12559,7 +12559,7 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
@@ -13534,7 +13534,7 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
@@ -14509,7 +14509,7 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
@@ -14834,7 +14834,7 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
@@ -14899,7 +14899,7 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
@@ -14964,7 +14964,7 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
@@ -15029,7 +15029,7 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
@@ -15224,7 +15224,7 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
@@ -15354,7 +15354,7 @@
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F230" t="inlineStr">
@@ -16199,7 +16199,7 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -16329,7 +16329,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -16589,7 +16589,7 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -17434,7 +17434,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -17564,7 +17564,7 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
@@ -17889,7 +17889,7 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
@@ -18344,7 +18344,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
@@ -18409,7 +18409,7 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
@@ -18734,7 +18734,7 @@
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F282" t="inlineStr">
@@ -19189,7 +19189,7 @@
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F289" t="inlineStr">
@@ -19514,7 +19514,7 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
@@ -19644,7 +19644,7 @@
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F296" t="inlineStr">
@@ -19949,7 +19949,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>507428-1009-CM26</t>
+          <t>1557-337-CM26</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -19969,22 +19969,22 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>61.979.210-6</t>
+          <t>61.606.309-k</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD CHILOE</t>
+          <t>SERVICIO SALUD ATACAMA HOSPITAL DE HUASCO</t>
         </is>
       </c>
       <c r="H301" t="inlineStr">
         <is>
-          <t>Los Lagos</t>
+          <t>Atacama</t>
         </is>
       </c>
       <c r="I301" t="inlineStr">
@@ -20008,13 +20008,13 @@
         </is>
       </c>
       <c r="M301" s="2" t="n">
-        <v>30443.92</v>
+        <v>18525.25</v>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>918434-349-CM26</t>
+          <t>507428-1009-CM26</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
@@ -20039,17 +20039,17 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t>61.980.680-8</t>
+          <t>61.979.210-6</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
         <is>
-          <t>MINISTERIO DE LA MUJER Y LA EQUIDAD DE GÉNERO</t>
+          <t>SERVICIO DE SALUD CHILOE</t>
         </is>
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -20073,13 +20073,13 @@
         </is>
       </c>
       <c r="M302" s="2" t="n">
-        <v>403.66</v>
+        <v>30443.92</v>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>3951-264-CM26</t>
+          <t>918434-349-CM26</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
@@ -20104,17 +20104,17 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>61.974.700-3</t>
+          <t>61.980.680-8</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
         <is>
-          <t>CONSULTORIO GENERAL URBANO VICTOR DOMINGO SILVA</t>
+          <t>MINISTERIO DE LA MUJER Y LA EQUIDAD DE GÉNERO</t>
         </is>
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>Aysén</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -20138,13 +20138,13 @@
         </is>
       </c>
       <c r="M303" s="2" t="n">
-        <v>11430.68</v>
+        <v>403.66</v>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>4293-42-CM26</t>
+          <t>3951-264-CM26</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
@@ -20164,22 +20164,22 @@
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t>60.706.069-k</t>
+          <t>61.974.700-3</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
         <is>
-          <t>CORPORACION DE FOMENTO DE LA PRODUCCION</t>
+          <t>CONSULTORIO GENERAL URBANO VICTOR DOMINGO SILVA</t>
         </is>
       </c>
       <c r="H304" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Aysén</t>
         </is>
       </c>
       <c r="I304" t="inlineStr">
@@ -20203,13 +20203,13 @@
         </is>
       </c>
       <c r="M304" s="2" t="n">
-        <v>1771.56</v>
+        <v>11430.68</v>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>5195-179-CM26</t>
+          <t>4293-42-CM26</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
@@ -20229,17 +20229,17 @@
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t>65.743.680-1</t>
+          <t>60.706.069-k</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>CORPORACION DE FOMENTO DE LA PRODUCCION</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
@@ -20268,13 +20268,13 @@
         </is>
       </c>
       <c r="M305" s="2" t="n">
-        <v>2143.39</v>
+        <v>1771.56</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>1557-337-CM26</t>
+          <t>5195-179-CM26</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
@@ -20299,17 +20299,17 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>61.606.309-k</t>
+          <t>65.743.680-1</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
         <is>
-          <t>SERVICIO SALUD ATACAMA HOSPITAL DE HUASCO</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>Atacama</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I306" t="inlineStr">
@@ -20333,13 +20333,13 @@
         </is>
       </c>
       <c r="M306" s="2" t="n">
-        <v>18525.25</v>
+        <v>2143.39</v>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>1413-945-CM26</t>
+          <t>1079516-1019-CM26</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -20359,32 +20359,32 @@
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t>61.004.098-5</t>
+          <t>61.979.360-9</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
         <is>
-          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>Los Lagos</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I307" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J307" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K307" t="inlineStr">
@@ -20398,7 +20398,7 @@
         </is>
       </c>
       <c r="M307" s="2" t="n">
-        <v>2634.58</v>
+        <v>15622.47</v>
       </c>
     </row>
     <row r="308">
@@ -20424,7 +20424,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -20489,7 +20489,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -20554,7 +20554,7 @@
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F310" t="inlineStr">
@@ -20794,7 +20794,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>1079516-1019-CM26</t>
+          <t>1079516-1018-CM26</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -20814,7 +20814,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -20853,7 +20853,7 @@
         </is>
       </c>
       <c r="M314" s="2" t="n">
-        <v>15622.47</v>
+        <v>40847.73</v>
       </c>
     </row>
     <row r="315">
@@ -20879,7 +20879,7 @@
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F315" t="inlineStr">
@@ -21054,7 +21054,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>1079516-1018-CM26</t>
+          <t>3787-57-CM26</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -21079,7 +21079,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t>61.979.360-9</t>
+          <t>60.505.000-K</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -21089,17 +21089,17 @@
       </c>
       <c r="H318" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I318" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -21113,13 +21113,13 @@
         </is>
       </c>
       <c r="M318" s="2" t="n">
-        <v>40847.73</v>
+        <v>10586.77</v>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>3787-57-CM26</t>
+          <t>1413-945-CM26</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -21144,17 +21144,17 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>60.505.000-K</t>
+          <t>61.004.098-5</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>DIRECCION GENERAL DE GENDARMERIA DE CHIL</t>
         </is>
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Los Lagos</t>
         </is>
       </c>
       <c r="I319" t="inlineStr">
@@ -21178,13 +21178,13 @@
         </is>
       </c>
       <c r="M319" s="2" t="n">
-        <v>10586.77</v>
+        <v>2634.58</v>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>1079516-1017-CM26</t>
+          <t>1079516-1016-CM26</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -21204,7 +21204,7 @@
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F320" t="inlineStr">
@@ -21243,13 +21243,13 @@
         </is>
       </c>
       <c r="M320" s="2" t="n">
-        <v>8339.299999999999</v>
+        <v>11606.31</v>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>1075337-9903-CM26</t>
+          <t>1079516-1017-CM26</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -21274,27 +21274,27 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t>61.602.222-9</t>
+          <t>61.979.360-9</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD ARAUCANIA NORTE HOSPITAL DE ANGOL</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H321" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I321" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
         </is>
       </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.032.107-9</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
@@ -21308,13 +21308,13 @@
         </is>
       </c>
       <c r="M321" s="2" t="n">
-        <v>36191.59</v>
+        <v>8339.299999999999</v>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>2547-221-CM26</t>
+          <t>1075337-9903-CM26</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
@@ -21334,17 +21334,17 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>61.955.000-5</t>
+          <t>61.602.222-9</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
         <is>
-          <t>I MUNICIPALIDAD DE PADRE LAS CASAS</t>
+          <t>SERVICIO DE SALUD ARAUCANIA NORTE HOSPITAL DE ANGOL</t>
         </is>
       </c>
       <c r="H322" t="inlineStr">
@@ -21354,17 +21354,17 @@
       </c>
       <c r="I322" t="inlineStr">
         <is>
-          <t>SOCIEDAD DE CONFECCIONES CLER LIMITADA</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J322" t="inlineStr">
         <is>
-          <t>76.045.081-2</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="L322" t="inlineStr">
@@ -21373,13 +21373,13 @@
         </is>
       </c>
       <c r="M322" s="2" t="n">
-        <v>1543.11</v>
+        <v>36191.59</v>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>3374-126-CM26</t>
+          <t>2547-221-CM26</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
@@ -21399,37 +21399,37 @@
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>61.101.006-0</t>
+          <t>61.955.000-5</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>I MUNICIPALIDAD DE PADRE LAS CASAS</t>
         </is>
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SOCIEDAD DE CONFECCIONES CLER LIMITADA</t>
         </is>
       </c>
       <c r="J323" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>76.045.081-2</t>
         </is>
       </c>
       <c r="K323" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="L323" t="inlineStr">
@@ -21438,13 +21438,13 @@
         </is>
       </c>
       <c r="M323" s="2" t="n">
-        <v>184.49</v>
+        <v>1543.11</v>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>2080-9855-CM26</t>
+          <t>3374-126-CM26</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
@@ -21464,17 +21464,17 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t>61.602.138-9</t>
+          <t>61.101.006-0</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD DEL LIBERTADOR B O'HIGGINS HOSPITAL REG RANCAGUA</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H324" t="inlineStr">
@@ -21503,13 +21503,13 @@
         </is>
       </c>
       <c r="M324" s="2" t="n">
-        <v>11924.84</v>
+        <v>184.49</v>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>4146-55-CM26</t>
+          <t>2080-9855-CM26</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -21529,22 +21529,22 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>60.505.000-K</t>
+          <t>61.602.138-9</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>SERVICIO DE SALUD DEL LIBERTADOR B O'HIGGINS HOSPITAL REG RANCAGUA</t>
         </is>
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I325" t="inlineStr">
@@ -21568,7 +21568,7 @@
         </is>
       </c>
       <c r="M325" s="2" t="n">
-        <v>14785.89</v>
+        <v>11924.84</v>
       </c>
     </row>
     <row r="326">
@@ -21594,7 +21594,7 @@
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F326" t="inlineStr">
@@ -21639,7 +21639,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>1070329-276-CM26</t>
+          <t>3434-90-CM26</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -21664,17 +21664,17 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t>61.980.370-1</t>
+          <t>60.505.522-2</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
         <is>
-          <t>CESFAM LIRQUEN</t>
+          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
         </is>
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>Biobío</t>
+          <t>Araucanía</t>
         </is>
       </c>
       <c r="I327" t="inlineStr">
@@ -21698,13 +21698,13 @@
         </is>
       </c>
       <c r="M327" s="2" t="n">
-        <v>14728.76</v>
+        <v>35092.36</v>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>5251-878-CM26</t>
+          <t>1070329-276-CM26</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -21724,22 +21724,22 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>70.729.100-1</t>
+          <t>61.980.370-1</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
         <is>
-          <t>UNIVERSIDAD TECNOLOGICA METROPOLITANA</t>
+          <t>CESFAM LIRQUEN</t>
         </is>
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Biobío</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
@@ -21763,13 +21763,13 @@
         </is>
       </c>
       <c r="M328" s="2" t="n">
-        <v>7758.53</v>
+        <v>14728.76</v>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>1079516-1015-CM26</t>
+          <t>5251-878-CM26</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -21794,27 +21794,27 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t>61.979.360-9</t>
+          <t>70.729.100-1</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
         <is>
-          <t>DIRECCION DE LOGISTICA DE CARABINEROS</t>
+          <t>UNIVERSIDAD TECNOLOGICA METROPOLITANA</t>
         </is>
       </c>
       <c r="H329" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I329" t="inlineStr">
         <is>
-          <t>FDD INNOVACION &amp; CRECIMIENTO S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>76.032.107-9</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -21828,13 +21828,13 @@
         </is>
       </c>
       <c r="M329" s="2" t="n">
-        <v>29970.25</v>
+        <v>7758.53</v>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>1079516-1016-CM26</t>
+          <t>1079516-1015-CM26</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
@@ -21854,7 +21854,7 @@
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F330" t="inlineStr">
@@ -21893,13 +21893,13 @@
         </is>
       </c>
       <c r="M330" s="2" t="n">
-        <v>11606.31</v>
+        <v>29970.25</v>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>3434-90-CM26</t>
+          <t>4146-55-CM26</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -21924,7 +21924,7 @@
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t>60.505.522-2</t>
+          <t>60.505.000-K</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
@@ -21934,7 +21934,7 @@
       </c>
       <c r="H331" t="inlineStr">
         <is>
-          <t>Araucanía</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I331" t="inlineStr">
@@ -21958,7 +21958,7 @@
         </is>
       </c>
       <c r="M331" s="2" t="n">
-        <v>35092.36</v>
+        <v>14785.89</v>
       </c>
     </row>
     <row r="332">
@@ -21984,7 +21984,7 @@
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F332" t="inlineStr">
@@ -22179,7 +22179,7 @@
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F335" t="inlineStr">
@@ -22309,7 +22309,7 @@
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F337" t="inlineStr">
@@ -22354,7 +22354,7 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>463-83-CM26</t>
+          <t>889473-1764-CM26</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
@@ -22374,22 +22374,22 @@
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t>71.294.800-0</t>
+          <t>61.980.530-5</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
         <is>
-          <t>CENTRO DE INFORMACION DE RECURSOS NATURALES</t>
+          <t>UNIVERSIDAD DE O'HIGGINS</t>
         </is>
       </c>
       <c r="H338" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>O'Higgins</t>
         </is>
       </c>
       <c r="I338" t="inlineStr">
@@ -22413,7 +22413,7 @@
         </is>
       </c>
       <c r="M338" s="2" t="n">
-        <v>17810.53</v>
+        <v>7130.95</v>
       </c>
     </row>
     <row r="339">
@@ -22634,7 +22634,7 @@
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F342" t="inlineStr">
@@ -22679,7 +22679,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>889473-1764-CM26</t>
+          <t>1057496-1746-CM26</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -22699,22 +22699,22 @@
       </c>
       <c r="E343" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t>61.980.530-5</t>
+          <t>61.608.105-5</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
         <is>
-          <t>UNIVERSIDAD DE O'HIGGINS</t>
+          <t>SERVICIO DE SALUD SUR HOSPITAL SAN LUIS</t>
         </is>
       </c>
       <c r="H343" t="inlineStr">
         <is>
-          <t>O'Higgins</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I343" t="inlineStr">
@@ -22738,13 +22738,13 @@
         </is>
       </c>
       <c r="M343" s="2" t="n">
-        <v>7130.95</v>
+        <v>5812.09</v>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>1057496-1746-CM26</t>
+          <t>463-83-CM26</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -22764,17 +22764,17 @@
       </c>
       <c r="E344" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t>61.608.105-5</t>
+          <t>71.294.800-0</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
         <is>
-          <t>SERVICIO DE SALUD SUR HOSPITAL SAN LUIS</t>
+          <t>CENTRO DE INFORMACION DE RECURSOS NATURALES</t>
         </is>
       </c>
       <c r="H344" t="inlineStr">
@@ -22803,7 +22803,7 @@
         </is>
       </c>
       <c r="M344" s="2" t="n">
-        <v>5812.09</v>
+        <v>17810.53</v>
       </c>
     </row>
     <row r="345">
@@ -22829,7 +22829,7 @@
       </c>
       <c r="E345" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F345" t="inlineStr">
@@ -22894,7 +22894,7 @@
       </c>
       <c r="E346" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F346" t="inlineStr">
@@ -23024,7 +23024,7 @@
       </c>
       <c r="E348" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F348" t="inlineStr">
@@ -23089,7 +23089,7 @@
       </c>
       <c r="E349" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F349" t="inlineStr">
@@ -23219,7 +23219,7 @@
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F351" t="inlineStr">
@@ -23284,7 +23284,7 @@
       </c>
       <c r="E352" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F352" t="inlineStr">
@@ -23349,7 +23349,7 @@
       </c>
       <c r="E353" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F353" t="inlineStr">
@@ -23414,7 +23414,7 @@
       </c>
       <c r="E354" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F354" t="inlineStr">
@@ -23674,7 +23674,7 @@
       </c>
       <c r="E358" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F358" t="inlineStr">
@@ -23804,7 +23804,7 @@
       </c>
       <c r="E360" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F360" t="inlineStr">
@@ -23934,7 +23934,7 @@
       </c>
       <c r="E362" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F362" t="inlineStr">
@@ -23999,7 +23999,7 @@
       </c>
       <c r="E363" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F363" t="inlineStr">
@@ -24129,7 +24129,7 @@
       </c>
       <c r="E365" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F365" t="inlineStr">
@@ -24194,7 +24194,7 @@
       </c>
       <c r="E366" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F366" t="inlineStr">
@@ -24454,7 +24454,7 @@
       </c>
       <c r="E370" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F370" t="inlineStr">
@@ -24649,7 +24649,7 @@
       </c>
       <c r="E373" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F373" t="inlineStr">
@@ -24714,7 +24714,7 @@
       </c>
       <c r="E374" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F374" t="inlineStr">
@@ -24824,7 +24824,7 @@
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>1368-68-CM26</t>
+          <t>1099899-151-CM26</t>
         </is>
       </c>
       <c r="B376" t="inlineStr">
@@ -24844,22 +24844,22 @@
       </c>
       <c r="E376" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F376" t="inlineStr">
         <is>
-          <t>75.980.060-5</t>
+          <t>62.000.630-0</t>
         </is>
       </c>
       <c r="G376" t="inlineStr">
         <is>
-          <t>CORPORACION DE FOMENTO DE LA PRODUCCION</t>
+          <t>CENTRO SALUD MENTAL COMUNITARIA LOS ANDES</t>
         </is>
       </c>
       <c r="H376" t="inlineStr">
         <is>
-          <t>Metropolitana</t>
+          <t>Valparaíso</t>
         </is>
       </c>
       <c r="I376" t="inlineStr">
@@ -24883,7 +24883,7 @@
         </is>
       </c>
       <c r="M376" s="2" t="n">
-        <v>1142.96</v>
+        <v>6809.39</v>
       </c>
     </row>
     <row r="377">
@@ -24909,7 +24909,7 @@
       </c>
       <c r="E377" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F377" t="inlineStr">
@@ -24954,7 +24954,7 @@
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>1099899-151-CM26</t>
+          <t>1099899-150-CM26</t>
         </is>
       </c>
       <c r="B378" t="inlineStr">
@@ -25013,7 +25013,7 @@
         </is>
       </c>
       <c r="M378" s="2" t="n">
-        <v>6809.39</v>
+        <v>1289.35</v>
       </c>
     </row>
     <row r="379">
@@ -25084,7 +25084,7 @@
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>812261-1403-CM26</t>
+          <t>4388-102-CM26</t>
         </is>
       </c>
       <c r="B380" t="inlineStr">
@@ -25104,17 +25104,17 @@
       </c>
       <c r="E380" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F380" t="inlineStr">
         <is>
-          <t>65.075.485-9</t>
+          <t>60.511.000-2</t>
         </is>
       </c>
       <c r="G380" t="inlineStr">
         <is>
-          <t>HOSPITAL CLINICO METROPOLITANO DE LA FLORIDA DOCTORA ELOISA DIAZ</t>
+          <t>SUBSECRETARIA DEL INTERIOR</t>
         </is>
       </c>
       <c r="H380" t="inlineStr">
@@ -25124,12 +25124,12 @@
       </c>
       <c r="I380" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J380" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K380" t="inlineStr">
@@ -25143,7 +25143,7 @@
         </is>
       </c>
       <c r="M380" s="2" t="n">
-        <v>30933.78</v>
+        <v>159.99</v>
       </c>
     </row>
     <row r="381">
@@ -25169,7 +25169,7 @@
       </c>
       <c r="E381" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F381" t="inlineStr">
@@ -25234,7 +25234,7 @@
       </c>
       <c r="E382" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F382" t="inlineStr">
@@ -25364,7 +25364,7 @@
       </c>
       <c r="E384" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F384" t="inlineStr">
@@ -25494,7 +25494,7 @@
       </c>
       <c r="E386" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F386" t="inlineStr">
@@ -25539,7 +25539,7 @@
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>721703-464-CM26</t>
+          <t>812261-1403-CM26</t>
         </is>
       </c>
       <c r="B387" t="inlineStr">
@@ -25564,12 +25564,12 @@
       </c>
       <c r="F387" t="inlineStr">
         <is>
-          <t>61.980.230-6</t>
+          <t>65.075.485-9</t>
         </is>
       </c>
       <c r="G387" t="inlineStr">
         <is>
-          <t>AGENCIA DE CALIDAD DE LA EDUCACION</t>
+          <t>HOSPITAL CLINICO METROPOLITANO DE LA FLORIDA DOCTORA ELOISA DIAZ</t>
         </is>
       </c>
       <c r="H387" t="inlineStr">
@@ -25579,12 +25579,12 @@
       </c>
       <c r="I387" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J387" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K387" t="inlineStr">
@@ -25598,13 +25598,13 @@
         </is>
       </c>
       <c r="M387" s="2" t="n">
-        <v>1772.36</v>
+        <v>30933.78</v>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>5003-40-CM26</t>
+          <t>721703-464-CM26</t>
         </is>
       </c>
       <c r="B388" t="inlineStr">
@@ -25629,12 +25629,12 @@
       </c>
       <c r="F388" t="inlineStr">
         <is>
-          <t>61.978.750-1</t>
+          <t>61.980.230-6</t>
         </is>
       </c>
       <c r="G388" t="inlineStr">
         <is>
-          <t>DIVISION LOGISTICA DEL EJERCITO</t>
+          <t>AGENCIA DE CALIDAD DE LA EDUCACION</t>
         </is>
       </c>
       <c r="H388" t="inlineStr">
@@ -25644,12 +25644,12 @@
       </c>
       <c r="I388" t="inlineStr">
         <is>
-          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
+          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
         </is>
       </c>
       <c r="J388" t="inlineStr">
         <is>
-          <t>96.556.930-8</t>
+          <t>96.781.350-8</t>
         </is>
       </c>
       <c r="K388" t="inlineStr">
@@ -25663,7 +25663,7 @@
         </is>
       </c>
       <c r="M388" s="2" t="n">
-        <v>819.39</v>
+        <v>1772.36</v>
       </c>
     </row>
     <row r="389">
@@ -25689,7 +25689,7 @@
       </c>
       <c r="E389" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F389" t="inlineStr">
@@ -26014,7 +26014,7 @@
       </c>
       <c r="E394" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F394" t="inlineStr">
@@ -26059,7 +26059,7 @@
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>4388-102-CM26</t>
+          <t>5003-40-CM26</t>
         </is>
       </c>
       <c r="B395" t="inlineStr">
@@ -26084,12 +26084,12 @@
       </c>
       <c r="F395" t="inlineStr">
         <is>
-          <t>60.511.000-2</t>
+          <t>61.978.750-1</t>
         </is>
       </c>
       <c r="G395" t="inlineStr">
         <is>
-          <t>SUBSECRETARIA DEL INTERIOR</t>
+          <t>DIVISION LOGISTICA DEL EJERCITO</t>
         </is>
       </c>
       <c r="H395" t="inlineStr">
@@ -26099,12 +26099,12 @@
       </c>
       <c r="I395" t="inlineStr">
         <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
+          <t>SODEXO SOLUCIONES DE MOTIVACION CHILE S.A.</t>
         </is>
       </c>
       <c r="J395" t="inlineStr">
         <is>
-          <t>96.781.350-8</t>
+          <t>96.556.930-8</t>
         </is>
       </c>
       <c r="K395" t="inlineStr">
@@ -26118,13 +26118,13 @@
         </is>
       </c>
       <c r="M395" s="2" t="n">
-        <v>159.99</v>
+        <v>819.39</v>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>1099899-150-CM26</t>
+          <t>761-308-CM26</t>
         </is>
       </c>
       <c r="B396" t="inlineStr">
@@ -26144,22 +26144,22 @@
       </c>
       <c r="E396" t="inlineStr">
         <is>
-          <t>Recepcion Conforme</t>
+          <t>Aceptada</t>
         </is>
       </c>
       <c r="F396" t="inlineStr">
         <is>
-          <t>62.000.630-0</t>
+          <t>60.515.000-4</t>
         </is>
       </c>
       <c r="G396" t="inlineStr">
         <is>
-          <t>CENTRO SALUD MENTAL COMUNITARIA LOS ANDES</t>
+          <t>SUBSECRETARIA DE DESARROLLO REGIONAL Y ADMINISTRATIVO</t>
         </is>
       </c>
       <c r="H396" t="inlineStr">
         <is>
-          <t>Valparaíso</t>
+          <t>Metropolitana</t>
         </is>
       </c>
       <c r="I396" t="inlineStr">
@@ -26183,71 +26183,6 @@
         </is>
       </c>
       <c r="M396" s="2" t="n">
-        <v>1289.35</v>
-      </c>
-    </row>
-    <row r="397">
-      <c r="A397" t="inlineStr">
-        <is>
-          <t>761-308-CM26</t>
-        </is>
-      </c>
-      <c r="B397" t="inlineStr">
-        <is>
-          <t>2239-1-LR26</t>
-        </is>
-      </c>
-      <c r="C397" t="inlineStr">
-        <is>
-          <t>sep-2026</t>
-        </is>
-      </c>
-      <c r="D397" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E397" t="inlineStr">
-        <is>
-          <t>Aceptada</t>
-        </is>
-      </c>
-      <c r="F397" t="inlineStr">
-        <is>
-          <t>60.515.000-4</t>
-        </is>
-      </c>
-      <c r="G397" t="inlineStr">
-        <is>
-          <t>SUBSECRETARIA DE DESARROLLO REGIONAL Y ADMINISTRATIVO</t>
-        </is>
-      </c>
-      <c r="H397" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
-      <c r="I397" t="inlineStr">
-        <is>
-          <t>EDENRED CHILE SOCIEDAD ANONIMA</t>
-        </is>
-      </c>
-      <c r="J397" t="inlineStr">
-        <is>
-          <t>96.781.350-8</t>
-        </is>
-      </c>
-      <c r="K397" t="inlineStr">
-        <is>
-          <t>Metropolitana</t>
-        </is>
-      </c>
-      <c r="L397" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="M397" s="2" t="n">
         <v>1854.79</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Seguro pasa al nuevo convenio 2239-7-LR26 (el 2239-12-LR23 venció el 25-10-2026) y datos transaccionales al 26-10-2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/oc-mensuales/administracion-y-entrega-de-beneficios/sep-2026.xlsx
+++ b/docs/oc-mensuales/administracion-y-entrega-de-beneficios/sep-2026.xlsx
@@ -17694,7 +17694,7 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
@@ -17824,7 +17824,7 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Aceptada</t>
+          <t>Recepcion Conforme</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">

</xml_diff>